<commit_message>
Running through final data after merge
</commit_message>
<xml_diff>
--- a/dcor-wpac-final/qaqc.full-final-dataset.xlsx
+++ b/dcor-wpac-final/qaqc.full-final-dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aonoufriou/Documents/GitHub/Turtle_GTseq_SNPs/dcor-wpac-final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23EBA169-FEC5-D543-833F-542CFE68C855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4336584-1F6E-2C41-93A4-6CAC6A8EE9A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="920" windowWidth="34120" windowHeight="21260" firstSheet="1" activeTab="1" xr2:uid="{2F8F4325-B2C8-0F46-B2F3-681D9E737D6A}"/>
+    <workbookView xWindow="160" yWindow="920" windowWidth="17060" windowHeight="21260" activeTab="1" xr2:uid="{2F8F4325-B2C8-0F46-B2F3-681D9E737D6A}"/>
   </bookViews>
   <sheets>
     <sheet name="sample_data" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
     <sheet name="wreps_mismatches" sheetId="6" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">labels_zpad_merged!$A$1:$C$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">labels_zpad_merged!$E$1:$E$383</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sample_data!$A$1:$CU$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'wreps_dup-check'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'wreps_genos-to-check'!$A$1:$O$1</definedName>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10272" uniqueCount="1808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10268" uniqueCount="1813">
   <si>
     <t>z0006796_mapped2ref.sam</t>
   </si>
@@ -5232,9 +5232,6 @@
     <t>z0012509_merged.sam</t>
   </si>
   <si>
-    <t>z0012514_merged.sam</t>
-  </si>
-  <si>
     <t>z0012519_merged.sam</t>
   </si>
   <si>
@@ -5476,13 +5473,31 @@
   </si>
   <si>
     <t xml:space="preserve">Will merge and run the script again. </t>
+  </si>
+  <si>
+    <t>Also need to fix these duplicates:</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -12504 and 12514: Keep 12504, drop 12514</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -26457 and 40945: merge and call 26547</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -26450 and 40943: merge and call 26450</t>
+  </si>
+  <si>
+    <t>One individual with &gt;70% homozygosity: z0062726</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -Will leave for now</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -5540,8 +5555,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5566,6 +5588,11 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -5576,10 +5603,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -5617,11 +5645,16 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5689,6 +5722,24 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -40267,22 +40318,22 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D331:D1048576 E326:E330">
-    <cfRule type="duplicateValues" dxfId="5" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1">
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E98">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E99:E325">
-    <cfRule type="duplicateValues" dxfId="2" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="O274:U325">
-    <cfRule type="duplicateValues" dxfId="1" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="7"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -41333,7 +41384,7 @@
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>1800</v>
+        <v>1799</v>
       </c>
       <c r="C23" t="s">
         <v>473</v>
@@ -41369,7 +41420,7 @@
         <v>3</v>
       </c>
       <c r="N23" t="s">
-        <v>1801</v>
+        <v>1800</v>
       </c>
       <c r="O23" t="s">
         <v>1666</v>
@@ -41817,7 +41868,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>1800</v>
+        <v>1799</v>
       </c>
       <c r="B23" t="s">
         <v>473</v>
@@ -42762,7 +42813,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C1F9018-7BD2-E14A-A0D9-372512C3AE0B}">
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:H115"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
@@ -43090,7 +43141,7 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>1773</v>
+        <v>1772</v>
       </c>
     </row>
     <row r="64" spans="1:8" s="20" customFormat="1" x14ac:dyDescent="0.2">
@@ -43107,10 +43158,10 @@
         <v>1642</v>
       </c>
       <c r="E64" s="19" t="s">
-        <v>1774</v>
+        <v>1773</v>
       </c>
       <c r="F64" s="18" t="s">
-        <v>1777</v>
+        <v>1776</v>
       </c>
       <c r="G64" s="18"/>
       <c r="H64" s="18"/>
@@ -43129,10 +43180,10 @@
         <v>1157</v>
       </c>
       <c r="E65" s="17" t="s">
-        <v>1775</v>
+        <v>1774</v>
       </c>
       <c r="F65" s="17" t="s">
-        <v>1778</v>
+        <v>1777</v>
       </c>
       <c r="G65" s="13"/>
       <c r="H65" s="14"/>
@@ -43151,10 +43202,10 @@
         <v>1157</v>
       </c>
       <c r="E66" s="16" t="s">
-        <v>1776</v>
+        <v>1775</v>
       </c>
       <c r="F66" s="16" t="s">
-        <v>1778</v>
+        <v>1777</v>
       </c>
       <c r="G66" s="10"/>
       <c r="H66" s="12"/>
@@ -43173,10 +43224,10 @@
         <v>1157</v>
       </c>
       <c r="E67" s="16" t="s">
-        <v>1776</v>
+        <v>1775</v>
       </c>
       <c r="F67" s="16" t="s">
-        <v>1778</v>
+        <v>1777</v>
       </c>
       <c r="G67" s="10"/>
       <c r="H67" s="12"/>
@@ -43195,10 +43246,10 @@
         <v>1364</v>
       </c>
       <c r="E68" s="17" t="s">
-        <v>1775</v>
+        <v>1774</v>
       </c>
       <c r="F68" s="17" t="s">
-        <v>1778</v>
+        <v>1777</v>
       </c>
       <c r="G68" s="13"/>
       <c r="H68" s="14"/>
@@ -43217,10 +43268,10 @@
         <v>1364</v>
       </c>
       <c r="E69" s="17" t="s">
-        <v>1775</v>
+        <v>1774</v>
       </c>
       <c r="F69" s="17" t="s">
-        <v>1778</v>
+        <v>1777</v>
       </c>
       <c r="G69" s="13"/>
       <c r="H69" s="14"/>
@@ -43239,10 +43290,10 @@
         <v>1157</v>
       </c>
       <c r="E70" s="16" t="s">
-        <v>1775</v>
+        <v>1774</v>
       </c>
       <c r="F70" s="16" t="s">
-        <v>1778</v>
+        <v>1777</v>
       </c>
       <c r="G70" s="10"/>
       <c r="H70" s="12"/>
@@ -43254,137 +43305,206 @@
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="10" t="s">
-        <v>1779</v>
+        <v>1778</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>1780</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>1781</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>1782</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>1783</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>1784</v>
+        <v>1783</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>1785</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>1786</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>1787</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>1788</v>
+        <v>1787</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>1789</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>1790</v>
+        <v>1789</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>1791</v>
+        <v>1790</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>1792</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>1793</v>
+        <v>1792</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>1794</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>1795</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>1796</v>
+        <v>1795</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>1797</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
+        <v>1796</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
         <v>46002</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
+        <v>1801</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
         <v>1802</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
         <v>1803</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
         <v>1804</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
-        <v>1805</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104" s="1">
         <v>46007</v>
       </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="F104" s="21"/>
+      <c r="G104" s="21"/>
+      <c r="H104" s="21"/>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
+        <v>1805</v>
+      </c>
+      <c r="F105" s="21"/>
+      <c r="G105" s="22"/>
+      <c r="H105" s="21"/>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
         <v>1806</v>
       </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
+      <c r="F106" s="21"/>
+      <c r="G106" s="22"/>
+      <c r="H106" s="21"/>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
         <v>1807</v>
+      </c>
+      <c r="F107" s="21"/>
+      <c r="G107" s="22"/>
+      <c r="H107" s="21"/>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>1808</v>
+      </c>
+      <c r="F108" s="21"/>
+      <c r="G108" s="23"/>
+      <c r="H108" s="21"/>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>1809</v>
+      </c>
+      <c r="F109" s="21"/>
+      <c r="G109" s="22"/>
+      <c r="H109" s="21"/>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>1810</v>
+      </c>
+      <c r="F110" s="21"/>
+      <c r="G110" s="22"/>
+      <c r="H110" s="21"/>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F111" s="21"/>
+      <c r="G111" s="22"/>
+      <c r="H111" s="21"/>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A112" s="24">
+        <v>46008</v>
+      </c>
+      <c r="F112" s="21"/>
+      <c r="G112" s="21"/>
+      <c r="H112" s="21"/>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>1811</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A114">
+        <v>-0.71710529999999995</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>1812</v>
       </c>
     </row>
   </sheetData>
@@ -46971,7 +47091,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72C37A7F-AAE7-9247-9323-4F8ED210C5C3}">
-  <dimension ref="A1:C262"/>
+  <dimension ref="A1:C258"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
@@ -47354,7 +47474,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>1798</v>
+        <v>1797</v>
       </c>
       <c r="B35" t="s">
         <v>367</v>
@@ -47431,10 +47551,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>1726</v>
+        <v>55</v>
       </c>
       <c r="B42" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C42" t="s">
         <v>648</v>
@@ -47442,10 +47562,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>55</v>
+        <v>1798</v>
       </c>
       <c r="B43" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C43" t="s">
         <v>648</v>
@@ -47453,10 +47573,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>1799</v>
+        <v>57</v>
       </c>
       <c r="B44" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C44" t="s">
         <v>648</v>
@@ -47464,10 +47584,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B45" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C45" t="s">
         <v>648</v>
@@ -47475,10 +47595,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>58</v>
+        <v>1726</v>
       </c>
       <c r="B46" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C46" t="s">
         <v>648</v>
@@ -47489,7 +47609,7 @@
         <v>1727</v>
       </c>
       <c r="B47" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C47" t="s">
         <v>648</v>
@@ -47500,7 +47620,7 @@
         <v>1728</v>
       </c>
       <c r="B48" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="C48" t="s">
         <v>648</v>
@@ -47508,10 +47628,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>1729</v>
+        <v>65</v>
       </c>
       <c r="B49" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C49" t="s">
         <v>648</v>
@@ -47519,10 +47639,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B50" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C50" t="s">
         <v>648</v>
@@ -47530,10 +47650,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B51" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C51" t="s">
         <v>648</v>
@@ -47541,10 +47661,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B52" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C52" t="s">
         <v>648</v>
@@ -47552,10 +47672,10 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B53" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C53" t="s">
         <v>648</v>
@@ -47563,10 +47683,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>69</v>
+        <v>1729</v>
       </c>
       <c r="B54" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C54" t="s">
         <v>648</v>
@@ -47574,10 +47694,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>1730</v>
+        <v>73</v>
       </c>
       <c r="B55" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="C55" t="s">
         <v>648</v>
@@ -47585,10 +47705,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B56" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C56" t="s">
         <v>648</v>
@@ -47596,10 +47716,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>74</v>
+        <v>1730</v>
       </c>
       <c r="B57" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C57" t="s">
         <v>648</v>
@@ -47607,10 +47727,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>1731</v>
+        <v>77</v>
       </c>
       <c r="B58" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C58" t="s">
         <v>648</v>
@@ -47618,10 +47738,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B59" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C59" t="s">
         <v>648</v>
@@ -47629,10 +47749,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B60" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C60" t="s">
         <v>648</v>
@@ -47640,10 +47760,10 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B61" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C61" t="s">
         <v>648</v>
@@ -47651,10 +47771,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>80</v>
+        <v>1731</v>
       </c>
       <c r="B62" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C62" t="s">
         <v>648</v>
@@ -47665,7 +47785,7 @@
         <v>1732</v>
       </c>
       <c r="B63" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C63" t="s">
         <v>648</v>
@@ -47676,7 +47796,7 @@
         <v>1733</v>
       </c>
       <c r="B64" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C64" t="s">
         <v>648</v>
@@ -47684,10 +47804,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>1734</v>
+        <v>87</v>
       </c>
       <c r="B65" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="C65" t="s">
         <v>648</v>
@@ -47695,10 +47815,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>87</v>
+        <v>1734</v>
       </c>
       <c r="B66" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C66" t="s">
         <v>648</v>
@@ -47706,10 +47826,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>1735</v>
+        <v>90</v>
       </c>
       <c r="B67" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="C67" t="s">
         <v>648</v>
@@ -47717,10 +47837,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>90</v>
+        <v>1735</v>
       </c>
       <c r="B68" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C68" t="s">
         <v>648</v>
@@ -47728,10 +47848,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>1736</v>
+        <v>93</v>
       </c>
       <c r="B69" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C69" t="s">
         <v>648</v>
@@ -47739,10 +47859,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B70" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C70" t="s">
         <v>648</v>
@@ -47750,10 +47870,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B71" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C71" t="s">
         <v>648</v>
@@ -47761,10 +47881,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B72" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C72" t="s">
         <v>648</v>
@@ -47772,10 +47892,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B73" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C73" t="s">
         <v>648</v>
@@ -47783,10 +47903,10 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B74" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C74" t="s">
         <v>648</v>
@@ -47794,10 +47914,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B75" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C75" t="s">
         <v>648</v>
@@ -47805,10 +47925,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B76" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C76" t="s">
         <v>648</v>
@@ -47816,10 +47936,10 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B77" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C77" t="s">
         <v>648</v>
@@ -47827,10 +47947,10 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B78" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C78" t="s">
         <v>648</v>
@@ -47838,10 +47958,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B79" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C79" t="s">
         <v>648</v>
@@ -47849,10 +47969,10 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>103</v>
+        <v>1736</v>
       </c>
       <c r="B80" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C80" t="s">
         <v>648</v>
@@ -47860,10 +47980,10 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>1737</v>
+        <v>106</v>
       </c>
       <c r="B81" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C81" t="s">
         <v>648</v>
@@ -47871,10 +47991,10 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B82" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C82" t="s">
         <v>648</v>
@@ -47882,10 +48002,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B83" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C83" t="s">
         <v>648</v>
@@ -47893,10 +48013,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B84" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C84" t="s">
         <v>648</v>
@@ -47904,10 +48024,10 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B85" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C85" t="s">
         <v>648</v>
@@ -47915,10 +48035,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B86" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C86" t="s">
         <v>648</v>
@@ -47926,10 +48046,10 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B87" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C87" t="s">
         <v>648</v>
@@ -47937,10 +48057,10 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>112</v>
+        <v>1737</v>
       </c>
       <c r="B88" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C88" t="s">
         <v>648</v>
@@ -47948,10 +48068,10 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>1738</v>
+        <v>115</v>
       </c>
       <c r="B89" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C89" t="s">
         <v>648</v>
@@ -47959,10 +48079,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B90" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C90" t="s">
         <v>648</v>
@@ -47970,10 +48090,10 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B91" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="C91" t="s">
         <v>648</v>
@@ -47981,10 +48101,10 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>117</v>
+        <v>1738</v>
       </c>
       <c r="B92" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="C92" t="s">
         <v>648</v>
@@ -47992,10 +48112,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B93" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="C93" t="s">
         <v>648</v>
@@ -48003,10 +48123,10 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B94" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="C94" t="s">
         <v>648</v>
@@ -48014,10 +48134,10 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>1739</v>
+        <v>125</v>
       </c>
       <c r="B95" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="C95" t="s">
         <v>648</v>
@@ -48025,10 +48145,10 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B96" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C96" t="s">
         <v>648</v>
@@ -48036,10 +48156,10 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B97" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="C97" t="s">
         <v>648</v>
@@ -48047,10 +48167,10 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B98" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="C98" t="s">
         <v>648</v>
@@ -48058,10 +48178,10 @@
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>126</v>
+        <v>1739</v>
       </c>
       <c r="B99" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="C99" t="s">
         <v>648</v>
@@ -48069,10 +48189,10 @@
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B100" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="C100" t="s">
         <v>648</v>
@@ -48080,10 +48200,10 @@
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>128</v>
+        <v>1740</v>
       </c>
       <c r="B101" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="C101" t="s">
         <v>648</v>
@@ -48091,10 +48211,10 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>129</v>
+        <v>1741</v>
       </c>
       <c r="B102" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="C102" t="s">
         <v>648</v>
@@ -48102,10 +48222,10 @@
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>1740</v>
+        <v>1742</v>
       </c>
       <c r="B103" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="C103" t="s">
         <v>648</v>
@@ -48113,10 +48233,10 @@
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B104" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="C104" t="s">
         <v>648</v>
@@ -48124,10 +48244,10 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>1741</v>
+        <v>1743</v>
       </c>
       <c r="B105" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="C105" t="s">
         <v>648</v>
@@ -48135,10 +48255,10 @@
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>1742</v>
+        <v>1744</v>
       </c>
       <c r="B106" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="C106" t="s">
         <v>648</v>
@@ -48146,10 +48266,10 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>1743</v>
+        <v>1745</v>
       </c>
       <c r="B107" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="C107" t="s">
         <v>648</v>
@@ -48157,10 +48277,10 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B108" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="C108" t="s">
         <v>648</v>
@@ -48168,10 +48288,10 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>1744</v>
+        <v>147</v>
       </c>
       <c r="B109" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
       <c r="C109" t="s">
         <v>648</v>
@@ -48179,10 +48299,10 @@
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>1745</v>
+        <v>148</v>
       </c>
       <c r="B110" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="C110" t="s">
         <v>648</v>
@@ -48193,7 +48313,7 @@
         <v>1746</v>
       </c>
       <c r="B111" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="C111" t="s">
         <v>648</v>
@@ -48201,10 +48321,10 @@
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B112" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
       <c r="C112" t="s">
         <v>648</v>
@@ -48212,10 +48332,10 @@
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B113" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="C113" t="s">
         <v>648</v>
@@ -48223,10 +48343,10 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B114" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="C114" t="s">
         <v>648</v>
@@ -48234,10 +48354,10 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>1747</v>
+        <v>154</v>
       </c>
       <c r="B115" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="C115" t="s">
         <v>648</v>
@@ -48245,10 +48365,10 @@
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>151</v>
+        <v>1747</v>
       </c>
       <c r="B116" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="C116" t="s">
         <v>648</v>
@@ -48256,10 +48376,10 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B117" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="C117" t="s">
         <v>648</v>
@@ -48267,10 +48387,10 @@
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B118" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="C118" t="s">
         <v>648</v>
@@ -48278,10 +48398,10 @@
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B119" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="C119" t="s">
         <v>648</v>
@@ -48289,10 +48409,10 @@
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>1748</v>
+        <v>160</v>
       </c>
       <c r="B120" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="C120" t="s">
         <v>648</v>
@@ -48300,10 +48420,10 @@
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B121" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="C121" t="s">
         <v>648</v>
@@ -48311,10 +48431,10 @@
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B122" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="C122" t="s">
         <v>648</v>
@@ -48322,10 +48442,10 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B123" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="C123" t="s">
         <v>648</v>
@@ -48333,10 +48453,10 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B124" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="C124" t="s">
         <v>648</v>
@@ -48344,10 +48464,10 @@
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B125" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="C125" t="s">
         <v>648</v>
@@ -48355,10 +48475,10 @@
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>162</v>
+        <v>1748</v>
       </c>
       <c r="B126" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="C126" t="s">
         <v>648</v>
@@ -48366,10 +48486,10 @@
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B127" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="C127" t="s">
         <v>648</v>
@@ -48377,10 +48497,10 @@
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B128" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="C128" t="s">
         <v>648</v>
@@ -48388,10 +48508,10 @@
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B129" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="C129" t="s">
         <v>648</v>
@@ -48399,10 +48519,10 @@
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>1749</v>
+        <v>171</v>
       </c>
       <c r="B130" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="C130" t="s">
         <v>648</v>
@@ -48410,10 +48530,10 @@
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B131" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="C131" t="s">
         <v>648</v>
@@ -48421,10 +48541,10 @@
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B132" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="C132" t="s">
         <v>648</v>
@@ -48432,10 +48552,10 @@
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B133" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="C133" t="s">
         <v>648</v>
@@ -48443,10 +48563,10 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B134" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="C134" t="s">
         <v>648</v>
@@ -48454,10 +48574,10 @@
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>172</v>
+        <v>1749</v>
       </c>
       <c r="B135" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="C135" t="s">
         <v>648</v>
@@ -48465,10 +48585,10 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B136" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="C136" t="s">
         <v>648</v>
@@ -48476,10 +48596,10 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="B137" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="C137" t="s">
         <v>648</v>
@@ -48487,10 +48607,10 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B138" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="C138" t="s">
         <v>648</v>
@@ -48498,10 +48618,10 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>1750</v>
+        <v>181</v>
       </c>
       <c r="B139" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="C139" t="s">
         <v>648</v>
@@ -48509,10 +48629,10 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B140" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="C140" t="s">
         <v>648</v>
@@ -48520,10 +48640,10 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B141" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="C141" t="s">
         <v>648</v>
@@ -48531,10 +48651,10 @@
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B142" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="C142" t="s">
         <v>648</v>
@@ -48542,10 +48662,10 @@
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B143" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="C143" t="s">
         <v>648</v>
@@ -48553,10 +48673,10 @@
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B144" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="C144" t="s">
         <v>648</v>
@@ -48564,10 +48684,10 @@
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
-        <v>183</v>
+        <v>1750</v>
       </c>
       <c r="B145" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="C145" t="s">
         <v>648</v>
@@ -48575,10 +48695,10 @@
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
-        <v>184</v>
+        <v>1751</v>
       </c>
       <c r="B146" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="C146" t="s">
         <v>648</v>
@@ -48586,10 +48706,10 @@
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B147" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="C147" t="s">
         <v>648</v>
@@ -48597,10 +48717,10 @@
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
-        <v>186</v>
+        <v>1752</v>
       </c>
       <c r="B148" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="C148" t="s">
         <v>648</v>
@@ -48608,10 +48728,10 @@
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
-        <v>1751</v>
+        <v>1753</v>
       </c>
       <c r="B149" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="C149" t="s">
         <v>648</v>
@@ -48619,10 +48739,10 @@
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>1752</v>
+        <v>196</v>
       </c>
       <c r="B150" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
       <c r="C150" t="s">
         <v>648</v>
@@ -48630,10 +48750,10 @@
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
-        <v>191</v>
+        <v>1754</v>
       </c>
       <c r="B151" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="C151" t="s">
         <v>648</v>
@@ -48641,10 +48761,10 @@
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
-        <v>1753</v>
+        <v>199</v>
       </c>
       <c r="B152" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
       <c r="C152" t="s">
         <v>648</v>
@@ -48652,10 +48772,10 @@
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>1754</v>
+        <v>200</v>
       </c>
       <c r="B153" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C153" t="s">
         <v>648</v>
@@ -48663,10 +48783,10 @@
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="B154" t="s">
-        <v>520</v>
+        <v>525</v>
       </c>
       <c r="C154" t="s">
         <v>648</v>
@@ -48674,10 +48794,10 @@
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
-        <v>1755</v>
+        <v>202</v>
       </c>
       <c r="B155" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
       <c r="C155" t="s">
         <v>648</v>
@@ -48685,10 +48805,10 @@
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
-        <v>199</v>
+        <v>1755</v>
       </c>
       <c r="B156" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="C156" t="s">
         <v>648</v>
@@ -48696,10 +48816,10 @@
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="B157" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="C157" t="s">
         <v>648</v>
@@ -48707,10 +48827,10 @@
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B158" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="C158" t="s">
         <v>648</v>
@@ -48718,10 +48838,10 @@
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="B159" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C159" t="s">
         <v>648</v>
@@ -48729,10 +48849,10 @@
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>1756</v>
+        <v>209</v>
       </c>
       <c r="B160" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="C160" t="s">
         <v>648</v>
@@ -48740,10 +48860,10 @@
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B161" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="C161" t="s">
         <v>648</v>
@@ -48751,10 +48871,10 @@
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B162" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="C162" t="s">
         <v>648</v>
@@ -48762,10 +48882,10 @@
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B163" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="C163" t="s">
         <v>648</v>
@@ -48773,10 +48893,10 @@
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B164" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="C164" t="s">
         <v>648</v>
@@ -48784,10 +48904,10 @@
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>210</v>
+        <v>1756</v>
       </c>
       <c r="B165" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="C165" t="s">
         <v>648</v>
@@ -48795,10 +48915,10 @@
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="B166" t="s">
-        <v>535</v>
+        <v>540</v>
       </c>
       <c r="C166" t="s">
         <v>648</v>
@@ -48806,10 +48926,10 @@
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B167" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
       <c r="C167" t="s">
         <v>648</v>
@@ -48817,10 +48937,10 @@
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
-        <v>213</v>
+        <v>1757</v>
       </c>
       <c r="B168" t="s">
-        <v>537</v>
+        <v>542</v>
       </c>
       <c r="C168" t="s">
         <v>648</v>
@@ -48828,10 +48948,10 @@
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
-        <v>1757</v>
+        <v>1758</v>
       </c>
       <c r="B169" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="C169" t="s">
         <v>648</v>
@@ -48839,10 +48959,10 @@
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="B170" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C170" t="s">
         <v>648</v>
@@ -48850,10 +48970,10 @@
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
-        <v>217</v>
+        <v>1759</v>
       </c>
       <c r="B171" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="C171" t="s">
         <v>648</v>
@@ -48861,10 +48981,10 @@
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
-        <v>1758</v>
+        <v>1760</v>
       </c>
       <c r="B172" t="s">
-        <v>542</v>
+        <v>549</v>
       </c>
       <c r="C172" t="s">
         <v>648</v>
@@ -48872,10 +48992,10 @@
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
-        <v>1759</v>
+        <v>227</v>
       </c>
       <c r="B173" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="C173" t="s">
         <v>648</v>
@@ -48883,10 +49003,10 @@
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B174" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="C174" t="s">
         <v>648</v>
@@ -48894,10 +49014,10 @@
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
-        <v>1760</v>
+        <v>229</v>
       </c>
       <c r="B175" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="C175" t="s">
         <v>648</v>
@@ -48905,10 +49025,10 @@
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>1761</v>
+        <v>230</v>
       </c>
       <c r="B176" t="s">
-        <v>549</v>
+        <v>554</v>
       </c>
       <c r="C176" t="s">
         <v>648</v>
@@ -48916,10 +49036,10 @@
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B177" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="C177" t="s">
         <v>648</v>
@@ -48927,10 +49047,10 @@
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B178" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="C178" t="s">
         <v>648</v>
@@ -48938,10 +49058,10 @@
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B179" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="C179" t="s">
         <v>648</v>
@@ -48949,10 +49069,10 @@
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B180" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C180" t="s">
         <v>648</v>
@@ -48960,10 +49080,10 @@
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B181" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="C181" t="s">
         <v>648</v>
@@ -48971,10 +49091,10 @@
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B182" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="C182" t="s">
         <v>648</v>
@@ -48982,10 +49102,10 @@
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>1761</v>
       </c>
       <c r="B183" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="C183" t="s">
         <v>648</v>
@@ -48993,10 +49113,10 @@
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>1762</v>
       </c>
       <c r="B184" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="C184" t="s">
         <v>648</v>
@@ -49004,10 +49124,10 @@
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>1763</v>
       </c>
       <c r="B185" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="C185" t="s">
         <v>648</v>
@@ -49015,10 +49135,10 @@
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="B186" t="s">
-        <v>560</v>
+        <v>567</v>
       </c>
       <c r="C186" t="s">
         <v>648</v>
@@ -49026,10 +49146,10 @@
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>1762</v>
+        <v>1764</v>
       </c>
       <c r="B187" t="s">
-        <v>561</v>
+        <v>568</v>
       </c>
       <c r="C187" t="s">
         <v>648</v>
@@ -49037,10 +49157,10 @@
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>1763</v>
+        <v>246</v>
       </c>
       <c r="B188" t="s">
-        <v>563</v>
+        <v>570</v>
       </c>
       <c r="C188" t="s">
         <v>648</v>
@@ -49048,10 +49168,10 @@
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>1764</v>
+        <v>247</v>
       </c>
       <c r="B189" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="C189" t="s">
         <v>648</v>
@@ -49059,10 +49179,10 @@
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>243</v>
+        <v>1765</v>
       </c>
       <c r="B190" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="C190" t="s">
         <v>648</v>
@@ -49070,10 +49190,10 @@
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
-        <v>1765</v>
+        <v>250</v>
       </c>
       <c r="B191" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C191" t="s">
         <v>648</v>
@@ -49081,10 +49201,10 @@
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B192" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="C192" t="s">
         <v>648</v>
@@ -49092,10 +49212,10 @@
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B193" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="C193" t="s">
         <v>648</v>
@@ -49103,10 +49223,10 @@
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
-        <v>1766</v>
+        <v>253</v>
       </c>
       <c r="B194" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="C194" t="s">
         <v>648</v>
@@ -49114,10 +49234,10 @@
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B195" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C195" t="s">
         <v>648</v>
@@ -49125,10 +49245,10 @@
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
-        <v>251</v>
+        <v>1766</v>
       </c>
       <c r="B196" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="C196" t="s">
         <v>648</v>
@@ -49136,10 +49256,10 @@
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
-        <v>252</v>
+        <v>1767</v>
       </c>
       <c r="B197" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C197" t="s">
         <v>648</v>
@@ -49147,10 +49267,10 @@
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="B198" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="C198" t="s">
         <v>648</v>
@@ -49158,10 +49278,10 @@
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="B199" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="C199" t="s">
         <v>648</v>
@@ -49169,10 +49289,10 @@
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
-        <v>1767</v>
+        <v>261</v>
       </c>
       <c r="B200" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="C200" t="s">
         <v>648</v>
@@ -49183,7 +49303,7 @@
         <v>1768</v>
       </c>
       <c r="B201" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="C201" t="s">
         <v>648</v>
@@ -49191,10 +49311,10 @@
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="B202" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="C202" t="s">
         <v>648</v>
@@ -49202,10 +49322,10 @@
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
-        <v>260</v>
+        <v>1769</v>
       </c>
       <c r="B203" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
       <c r="C203" t="s">
         <v>648</v>
@@ -49213,10 +49333,10 @@
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B204" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="C204" t="s">
         <v>648</v>
@@ -49224,10 +49344,10 @@
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
-        <v>1769</v>
+        <v>268</v>
       </c>
       <c r="B205" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="C205" t="s">
         <v>648</v>
@@ -49235,10 +49355,10 @@
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
-        <v>264</v>
+        <v>1770</v>
       </c>
       <c r="B206" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
       <c r="C206" t="s">
         <v>648</v>
@@ -49246,10 +49366,10 @@
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
-        <v>1770</v>
+        <v>1771</v>
       </c>
       <c r="B207" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="C207" t="s">
         <v>648</v>
@@ -49257,10 +49377,10 @@
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="B208" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="C208" t="s">
         <v>648</v>
@@ -49268,10 +49388,10 @@
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="B209" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="C209" t="s">
         <v>648</v>
@@ -49279,10 +49399,10 @@
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
-        <v>1771</v>
+        <v>275</v>
       </c>
       <c r="B210" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="C210" t="s">
         <v>648</v>
@@ -49290,10 +49410,10 @@
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
-        <v>1772</v>
+        <v>276</v>
       </c>
       <c r="B211" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
       <c r="C211" t="s">
         <v>648</v>
@@ -49301,10 +49421,10 @@
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="B212" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="C212" t="s">
         <v>648</v>
@@ -49312,10 +49432,10 @@
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B213" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="C213" t="s">
         <v>648</v>
@@ -49323,10 +49443,10 @@
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B214" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="C214" t="s">
         <v>648</v>
@@ -49334,10 +49454,10 @@
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B215" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="C215" t="s">
         <v>648</v>
@@ -49345,10 +49465,10 @@
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B216" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="C216" t="s">
         <v>648</v>
@@ -49356,10 +49476,10 @@
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B217" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="C217" t="s">
         <v>648</v>
@@ -49367,10 +49487,10 @@
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="B218" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="C218" t="s">
         <v>648</v>
@@ -49378,10 +49498,10 @@
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B219" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C219" t="s">
         <v>648</v>
@@ -49389,10 +49509,10 @@
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B220" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="C220" t="s">
         <v>648</v>
@@ -49400,10 +49520,10 @@
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="B221" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="C221" t="s">
         <v>648</v>
@@ -49411,10 +49531,10 @@
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="B222" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="C222" t="s">
         <v>648</v>
@@ -49422,10 +49542,10 @@
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="B223" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="C223" t="s">
         <v>648</v>
@@ -49433,10 +49553,10 @@
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="B224" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="C224" t="s">
         <v>648</v>
@@ -49444,10 +49564,10 @@
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="B225" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="C225" t="s">
         <v>648</v>
@@ -49455,10 +49575,10 @@
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="B226" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="C226" t="s">
         <v>648</v>
@@ -49466,10 +49586,10 @@
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="B227" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="C227" t="s">
         <v>648</v>
@@ -49477,10 +49597,10 @@
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="B228" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="C228" t="s">
         <v>648</v>
@@ -49488,10 +49608,10 @@
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="B229" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="C229" t="s">
         <v>648</v>
@@ -49499,10 +49619,10 @@
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B230" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="C230" t="s">
         <v>648</v>
@@ -49510,10 +49630,10 @@
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="B231" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="C231" t="s">
         <v>648</v>
@@ -49521,10 +49641,10 @@
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="B232" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="C232" t="s">
         <v>648</v>
@@ -49532,10 +49652,10 @@
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="B233" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="C233" t="s">
         <v>648</v>
@@ -49543,10 +49663,10 @@
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="B234" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="C234" t="s">
         <v>648</v>
@@ -49554,10 +49674,10 @@
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="B235" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="C235" t="s">
         <v>648</v>
@@ -49565,10 +49685,10 @@
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="B236" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="C236" t="s">
         <v>648</v>
@@ -49576,10 +49696,10 @@
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="B237" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="C237" t="s">
         <v>648</v>
@@ -49587,10 +49707,10 @@
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="B238" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="C238" t="s">
         <v>648</v>
@@ -49598,10 +49718,10 @@
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="B239" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="C239" t="s">
         <v>648</v>
@@ -49609,10 +49729,10 @@
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B240" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="C240" t="s">
         <v>648</v>
@@ -49620,10 +49740,10 @@
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="B241" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="C241" t="s">
         <v>648</v>
@@ -49631,10 +49751,10 @@
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="B242" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="C242" t="s">
         <v>648</v>
@@ -49642,10 +49762,10 @@
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="B243" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="C243" t="s">
         <v>648</v>
@@ -49653,10 +49773,10 @@
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="B244" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="C244" t="s">
         <v>648</v>
@@ -49664,10 +49784,10 @@
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B245" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="C245" t="s">
         <v>648</v>
@@ -49675,10 +49795,10 @@
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="B246" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="C246" t="s">
         <v>648</v>
@@ -49686,10 +49806,10 @@
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="B247" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="C247" t="s">
         <v>648</v>
@@ -49697,10 +49817,10 @@
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="B248" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="C248" t="s">
         <v>648</v>
@@ -49708,10 +49828,10 @@
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="B249" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="C249" t="s">
         <v>648</v>
@@ -49719,10 +49839,10 @@
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="B250" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="C250" t="s">
         <v>648</v>
@@ -49730,10 +49850,10 @@
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="B251" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="C251" t="s">
         <v>648</v>
@@ -49741,10 +49861,10 @@
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="B252" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="C252" t="s">
         <v>648</v>
@@ -49752,10 +49872,10 @@
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="B253" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="C253" t="s">
         <v>648</v>
@@ -49763,10 +49883,10 @@
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B254" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="C254" t="s">
         <v>648</v>
@@ -49774,10 +49894,10 @@
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="B255" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="C255" t="s">
         <v>648</v>
@@ -49785,10 +49905,10 @@
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="B256" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="C256" t="s">
         <v>648</v>
@@ -49796,10 +49916,10 @@
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="B257" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="C257" t="s">
         <v>648</v>
@@ -49807,65 +49927,24 @@
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="B258" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="C258" t="s">
         <v>648</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A259" t="s">
-        <v>320</v>
-      </c>
-      <c r="B259" t="s">
-        <v>644</v>
-      </c>
-      <c r="C259" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A260" t="s">
-        <v>321</v>
-      </c>
-      <c r="B260" t="s">
-        <v>645</v>
-      </c>
-      <c r="C260" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A261" t="s">
-        <v>322</v>
-      </c>
-      <c r="B261" t="s">
-        <v>646</v>
-      </c>
-      <c r="C261" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A262" t="s">
-        <v>323</v>
-      </c>
-      <c r="B262" t="s">
-        <v>647</v>
-      </c>
-      <c r="C262" t="s">
-        <v>648</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:C323">
-    <sortCondition ref="B1:B323"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E1:E383">
+    <sortCondition sortBy="cellColor" ref="E1:E383" dxfId="8"/>
   </sortState>
+  <conditionalFormatting sqref="E1:E383 A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F1:F1048576 A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -49982,7 +50061,12 @@
         <f>"z00"&amp;E4</f>
         <v>z0012480</v>
       </c>
-      <c r="L4" s="10"/>
+      <c r="K4" s="10" t="s">
+        <v>356</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>453</v>
+      </c>
       <c r="M4" s="10"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -50021,6 +50105,7 @@
         <f t="shared" si="1"/>
         <v>z0012489</v>
       </c>
+      <c r="K6" s="10"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">

</xml_diff>

<commit_message>
Added cloneme repo and cleaned it up
</commit_message>
<xml_diff>
--- a/dcor-wpac-final/qaqc.full-final-dataset.xlsx
+++ b/dcor-wpac-final/qaqc.full-final-dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aonoufriou/Documents/GitHub/Turtle_GTseq_SNPs/dcor-wpac-final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D606D1A-D47B-4549-A525-6F28F0C20EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE52179B-B6EA-874E-BF6B-4BBAFBE73AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="17280" windowHeight="21680" activeTab="2" xr2:uid="{2F8F4325-B2C8-0F46-B2F3-681D9E737D6A}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15281" uniqueCount="1872">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15282" uniqueCount="1873">
   <si>
     <t>z0006796_mapped2ref.sam</t>
   </si>
@@ -5670,6 +5670,9 @@
   </si>
   <si>
     <t>Will drop locus 186 and keep 184 (better genotyping success rate)</t>
+  </si>
+  <si>
+    <t>Dropped loci as planned</t>
   </si>
 </sst>
 </file>
@@ -70940,7 +70943,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C1F9018-7BD2-E14A-A0D9-372512C3AE0B}">
-  <dimension ref="A1:L169"/>
+  <dimension ref="A1:L172"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" customWidth="1"/>
@@ -72134,6 +72137,16 @@
     <row r="169" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A169" s="10" t="s">
         <v>1871</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A170" s="10" t="s">
+        <v>1872</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A172" s="12">
+        <v>46044</v>
       </c>
     </row>
   </sheetData>

</xml_diff>